<commit_message>
feat: expand resource recommendations and radar data sync
</commit_message>
<xml_diff>
--- a/src/data/副本AI-Native读书雷达·资料共建.xlsx
+++ b/src/data/副本AI-Native读书雷达·资料共建.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10726"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B75EA930-5A17-6541-BA8C-4FAF604DDCBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C4A55B7-F395-6F4D-AD3A-B6110C13CCBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="推荐资料库" sheetId="2" r:id="rId1"/>
@@ -768,6 +768,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G89"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="35.33203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="4" max="4" width="40.6640625" customWidth="1"/>
+    <col min="6" max="6" width="39.5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">

</xml_diff>